<commit_message>
feat: basic distribution functios when generatin excel, and analyses/secuence bug corrections
</commit_message>
<xml_diff>
--- a/SupervisorMobility.API/DataAccess/Templates/Analysis Extra Template.xlsx
+++ b/SupervisorMobility.API/DataAccess/Templates/Analysis Extra Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27830"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ituriel\OneDrive\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8C6ACBC0-80F7-4B73-A2EA-2E55F4B35094}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{108133E8-6206-4D4B-95EA-E8AA1C0A1674}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="33210" yWindow="2520" windowWidth="30960" windowHeight="12225" xr2:uid="{BCFDEF49-20DD-4B13-9EF0-D1F3550AF258}"/>
+    <workbookView xWindow="52125" yWindow="6255" windowWidth="24825" windowHeight="12240" xr2:uid="{BCFDEF49-20DD-4B13-9EF0-D1F3550AF258}"/>
   </bookViews>
   <sheets>
     <sheet name="Name" sheetId="2" r:id="rId1"/>
@@ -667,7 +667,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="52">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -677,7 +677,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -718,16 +717,22 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="40" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -796,16 +801,16 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1161,105 +1166,105 @@
   </cols>
   <sheetData>
     <row r="3" spans="2:16" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B3" s="30" t="s">
+      <c r="B3" s="31" t="s">
         <v>14</v>
       </c>
-      <c r="C3" s="30"/>
-      <c r="D3" s="30"/>
-      <c r="E3" s="30"/>
-      <c r="F3" s="30"/>
-      <c r="G3" s="30"/>
-      <c r="H3" s="30"/>
-      <c r="I3" s="30"/>
-      <c r="J3" s="30"/>
+      <c r="C3" s="31"/>
+      <c r="D3" s="31"/>
+      <c r="E3" s="31"/>
+      <c r="F3" s="31"/>
+      <c r="G3" s="31"/>
+      <c r="H3" s="31"/>
+      <c r="I3" s="31"/>
+      <c r="J3" s="31"/>
     </row>
     <row r="4" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35"/>
     <row r="5" spans="2:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B5" s="46" t="s">
+      <c r="B5" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="C5" s="21" t="s">
         <v>13</v>
       </c>
-      <c r="D5" s="48"/>
-      <c r="E5" s="50" t="s">
+      <c r="D5" s="22"/>
+      <c r="E5" s="49" t="s">
         <v>12</v>
       </c>
-      <c r="F5" s="23" t="s">
+      <c r="F5" s="21" t="s">
         <v>11</v>
       </c>
-      <c r="G5" s="48"/>
-      <c r="H5" s="22" t="s">
+      <c r="G5" s="22"/>
+      <c r="H5" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="22"/>
-      <c r="J5" s="23" t="s">
+      <c r="I5" s="25"/>
+      <c r="J5" s="21" t="s">
         <v>9</v>
       </c>
-      <c r="K5" s="22"/>
-      <c r="L5" s="24"/>
-      <c r="M5" s="21" t="s">
+      <c r="K5" s="25"/>
+      <c r="L5" s="26"/>
+      <c r="M5" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="N5" s="20"/>
-      <c r="O5" s="20"/>
-      <c r="P5" s="20"/>
+      <c r="N5" s="19"/>
+      <c r="O5" s="19"/>
+      <c r="P5" s="19"/>
     </row>
     <row r="6" spans="2:16" ht="15" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B6" s="47"/>
-      <c r="C6" s="25"/>
-      <c r="D6" s="49"/>
-      <c r="E6" s="51"/>
-      <c r="F6" s="25"/>
-      <c r="G6" s="49"/>
-      <c r="H6" s="19" t="s">
+      <c r="B6" s="48"/>
+      <c r="C6" s="23"/>
+      <c r="D6" s="24"/>
+      <c r="E6" s="50"/>
+      <c r="F6" s="23"/>
+      <c r="G6" s="24"/>
+      <c r="H6" s="18" t="s">
         <v>7</v>
       </c>
-      <c r="I6" s="19" t="s">
+      <c r="I6" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="J6" s="25"/>
-      <c r="K6" s="26"/>
-      <c r="L6" s="27"/>
-      <c r="M6" s="18"/>
+      <c r="J6" s="23"/>
+      <c r="K6" s="27"/>
+      <c r="L6" s="28"/>
+      <c r="M6" s="17"/>
     </row>
     <row r="7" spans="2:16" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B7" s="17"/>
-      <c r="C7" s="33"/>
-      <c r="D7" s="34"/>
-      <c r="E7" s="16"/>
-      <c r="F7" s="35"/>
-      <c r="G7" s="36"/>
-      <c r="H7" s="15"/>
-      <c r="I7" s="14"/>
-      <c r="J7" s="33"/>
-      <c r="K7" s="37"/>
-      <c r="L7" s="38"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="34"/>
+      <c r="D7" s="35"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="36"/>
+      <c r="G7" s="37"/>
+      <c r="H7" s="14"/>
+      <c r="I7" s="13"/>
+      <c r="J7" s="34"/>
+      <c r="K7" s="38"/>
+      <c r="L7" s="39"/>
     </row>
     <row r="8" spans="2:16" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="13"/>
-      <c r="C8" s="39"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="12"/>
-      <c r="F8" s="41"/>
-      <c r="G8" s="42"/>
-      <c r="H8" s="11"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="39"/>
-      <c r="K8" s="43"/>
-      <c r="L8" s="44"/>
+      <c r="B8" s="12"/>
+      <c r="C8" s="40"/>
+      <c r="D8" s="41"/>
+      <c r="E8" s="11"/>
+      <c r="F8" s="42"/>
+      <c r="G8" s="43"/>
+      <c r="H8" s="10"/>
+      <c r="I8" s="9"/>
+      <c r="J8" s="40"/>
+      <c r="K8" s="44"/>
+      <c r="L8" s="45"/>
     </row>
     <row r="9" spans="2:16" ht="25.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="B9" s="9"/>
+      <c r="B9" s="8"/>
       <c r="C9" s="5"/>
       <c r="D9" s="5"/>
       <c r="E9" s="5"/>
       <c r="F9" s="5"/>
-      <c r="G9" s="8" t="s">
+      <c r="G9" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="H9" s="6"/>
-      <c r="I9" s="7"/>
+      <c r="H9" s="51"/>
+      <c r="I9" s="52"/>
       <c r="J9" s="6"/>
       <c r="K9" s="5"/>
       <c r="L9" s="4"/>
@@ -1269,30 +1274,31 @@
       <c r="L10" s="2"/>
     </row>
     <row r="11" spans="2:16" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B11" s="45" t="s">
+      <c r="B11" s="46" t="s">
         <v>4</v>
       </c>
-      <c r="C11" s="28"/>
-      <c r="D11" s="28"/>
+      <c r="C11" s="29"/>
+      <c r="D11" s="29"/>
       <c r="E11" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="F11" s="31" t="s">
+      <c r="F11" s="32" t="s">
         <v>2</v>
       </c>
-      <c r="G11" s="28"/>
-      <c r="H11" s="31" t="s">
+      <c r="G11" s="29"/>
+      <c r="H11" s="32" t="s">
         <v>1</v>
       </c>
-      <c r="I11" s="28"/>
-      <c r="J11" s="32"/>
-      <c r="K11" s="28" t="s">
+      <c r="I11" s="29"/>
+      <c r="J11" s="33"/>
+      <c r="K11" s="29" t="s">
         <v>0</v>
       </c>
-      <c r="L11" s="29"/>
+      <c r="L11" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="E5:E6"/>
     <mergeCell ref="F5:G6"/>
     <mergeCell ref="H5:I5"/>
     <mergeCell ref="J5:L6"/>
@@ -1309,7 +1315,6 @@
     <mergeCell ref="B11:D11"/>
     <mergeCell ref="B5:B6"/>
     <mergeCell ref="C5:D6"/>
-    <mergeCell ref="E5:E6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>